<commit_message>
Edit in excel 402
</commit_message>
<xml_diff>
--- a/402/402 LifeTable_10.xlsx
+++ b/402/402 LifeTable_10.xlsx
@@ -1,22 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\Lecture notes _2025\B.Stat 402\Practical\402 practical problem (Demography) By Anika\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F006AF7-5220-481A-8E98-B5FCC5026BE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="7" rupBuild="9303"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{6B8495CA-BC6C-41CE-A9C4-0EF3DB97FADD}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="19140" windowHeight="10140"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="145621"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="37">
   <si>
     <t>15-19</t>
   </si>
@@ -167,7 +161,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -538,22 +532,22 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68D40ADF-F83C-494C-A650-EEFA7B0809FF}">
-  <dimension ref="B2:H22"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B2:Q22"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="8.7265625" style="2"/>
-    <col min="5" max="5" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.7109375" style="2"/>
+    <col min="5" max="5" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" s="6" customFormat="1" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="2:17" s="6" customFormat="1" ht="18" x14ac:dyDescent="0.35">
       <c r="B2" s="5" t="s">
         <v>15</v>
       </c>
@@ -575,8 +569,29 @@
       <c r="H2" s="6" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="3" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="K2" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="M2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="N2" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="O2" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="P2" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q2" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B3" s="3">
         <v>0</v>
       </c>
@@ -602,8 +617,33 @@
         <f>G3/D3</f>
         <v>14.992316843386162</v>
       </c>
-    </row>
-    <row r="4" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="K3" s="3">
+        <v>0</v>
+      </c>
+      <c r="L3" s="1">
+        <v>0.08</v>
+      </c>
+      <c r="M3" s="4">
+        <v>100000</v>
+      </c>
+      <c r="N3" s="4">
+        <f>L3*M3</f>
+        <v>8000</v>
+      </c>
+      <c r="O3">
+        <f>(M3+M4)/2</f>
+        <v>96000</v>
+      </c>
+      <c r="P3">
+        <f>SUM(O3:O22)</f>
+        <v>1499231.6843386162</v>
+      </c>
+      <c r="Q3">
+        <f>P3/M3</f>
+        <v>14.992316843386162</v>
+      </c>
+    </row>
+    <row r="4" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B4" s="3">
         <v>1</v>
       </c>
@@ -630,8 +670,34 @@
         <f t="shared" ref="H4:H22" si="2">G4/D4</f>
         <v>15.252518308028437</v>
       </c>
-    </row>
-    <row r="5" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="K4" s="3">
+        <v>1</v>
+      </c>
+      <c r="L4" s="1">
+        <v>1.4E-2</v>
+      </c>
+      <c r="M4" s="4">
+        <f>M3-N3</f>
+        <v>92000</v>
+      </c>
+      <c r="N4" s="4">
+        <f>L4*M4</f>
+        <v>1288</v>
+      </c>
+      <c r="O4">
+        <f t="shared" ref="O4:O22" si="3">(M4+M5)/2</f>
+        <v>91356</v>
+      </c>
+      <c r="P4">
+        <f>SUM(O4:O23)</f>
+        <v>1403231.6843386162</v>
+      </c>
+      <c r="Q4">
+        <f t="shared" ref="Q4:Q22" si="4">P4/M4</f>
+        <v>15.252518308028437</v>
+      </c>
+    </row>
+    <row r="5" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B5" s="3">
         <v>2</v>
       </c>
@@ -658,8 +724,34 @@
         <f t="shared" si="2"/>
         <v>14.461986113619105</v>
       </c>
-    </row>
-    <row r="6" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="K5" s="3">
+        <v>2</v>
+      </c>
+      <c r="L5" s="1">
+        <v>1.2999999999999999E-2</v>
+      </c>
+      <c r="M5" s="4">
+        <f t="shared" ref="M5:M22" si="5">M4-N4</f>
+        <v>90712</v>
+      </c>
+      <c r="N5" s="4">
+        <f t="shared" ref="N4:N22" si="6">L5*M5</f>
+        <v>1179.2559999999999</v>
+      </c>
+      <c r="O5">
+        <f t="shared" si="3"/>
+        <v>90122.372000000003</v>
+      </c>
+      <c r="P5">
+        <f t="shared" ref="P4:P22" si="7">SUM(O5:O24)</f>
+        <v>1311875.6843386162</v>
+      </c>
+      <c r="Q5">
+        <f t="shared" si="4"/>
+        <v>14.461986113619105</v>
+      </c>
+    </row>
+    <row r="6" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B6" s="3">
         <v>3</v>
       </c>
@@ -686,8 +778,34 @@
         <f t="shared" si="2"/>
         <v>13.645882587253398</v>
       </c>
-    </row>
-    <row r="7" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="K6" s="3">
+        <v>3</v>
+      </c>
+      <c r="L6" s="1">
+        <v>1.2E-2</v>
+      </c>
+      <c r="M6" s="4">
+        <f t="shared" si="5"/>
+        <v>89532.744000000006</v>
+      </c>
+      <c r="N6" s="4">
+        <f t="shared" si="6"/>
+        <v>1074.392928</v>
+      </c>
+      <c r="O6">
+        <f t="shared" si="3"/>
+        <v>88995.547535999998</v>
+      </c>
+      <c r="P6">
+        <f t="shared" si="7"/>
+        <v>1221753.3123386162</v>
+      </c>
+      <c r="Q6">
+        <f t="shared" si="4"/>
+        <v>13.645882587253398</v>
+      </c>
+    </row>
+    <row r="7" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B7" s="3">
         <v>4</v>
       </c>
@@ -714,8 +832,34 @@
         <f t="shared" si="2"/>
         <v>12.80554917738198</v>
       </c>
-    </row>
-    <row r="8" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="K7" s="3">
+        <v>4</v>
+      </c>
+      <c r="L7" s="1">
+        <v>1.0999999999999999E-2</v>
+      </c>
+      <c r="M7" s="4">
+        <f t="shared" si="5"/>
+        <v>88458.351072000005</v>
+      </c>
+      <c r="N7" s="4">
+        <f t="shared" si="6"/>
+        <v>973.04186179199996</v>
+      </c>
+      <c r="O7">
+        <f t="shared" si="3"/>
+        <v>87971.830141104001</v>
+      </c>
+      <c r="P7">
+        <f t="shared" si="7"/>
+        <v>1132757.7648026161</v>
+      </c>
+      <c r="Q7">
+        <f t="shared" si="4"/>
+        <v>12.80554917738198</v>
+      </c>
+    </row>
+    <row r="8" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
         <v>13</v>
       </c>
@@ -742,8 +886,34 @@
         <f t="shared" si="2"/>
         <v>11.942415750639007</v>
       </c>
-    </row>
-    <row r="9" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="K8" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="L8" s="1">
+        <v>1.7999999999999999E-2</v>
+      </c>
+      <c r="M8" s="4">
+        <f t="shared" si="5"/>
+        <v>87485.309210208012</v>
+      </c>
+      <c r="N8" s="4">
+        <f t="shared" si="6"/>
+        <v>1574.7355657837441</v>
+      </c>
+      <c r="O8">
+        <f t="shared" si="3"/>
+        <v>86697.941427316138</v>
+      </c>
+      <c r="P8">
+        <f t="shared" si="7"/>
+        <v>1044785.934661512</v>
+      </c>
+      <c r="Q8">
+        <f t="shared" si="4"/>
+        <v>11.942415750639007</v>
+      </c>
+    </row>
+    <row r="9" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
         <v>14</v>
       </c>
@@ -751,7 +921,7 @@
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="D9" s="4">
-        <f t="shared" ref="D9:D22" si="3">D8-E8</f>
+        <f t="shared" ref="D9:D22" si="8">D8-E8</f>
         <v>85910.573644424265</v>
       </c>
       <c r="E9" s="4">
@@ -770,8 +940,34 @@
         <f t="shared" si="2"/>
         <v>11.152154532218951</v>
       </c>
-    </row>
-    <row r="10" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="K9" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="L9" s="1">
+        <v>6.0000000000000001E-3</v>
+      </c>
+      <c r="M9" s="4">
+        <f t="shared" si="5"/>
+        <v>85910.573644424265</v>
+      </c>
+      <c r="N9" s="4">
+        <f t="shared" si="6"/>
+        <v>515.46344186654562</v>
+      </c>
+      <c r="O9">
+        <f t="shared" si="3"/>
+        <v>85652.841923490982</v>
+      </c>
+      <c r="P9">
+        <f t="shared" si="7"/>
+        <v>958087.99323419598</v>
+      </c>
+      <c r="Q9">
+        <f t="shared" si="4"/>
+        <v>11.152154532218951</v>
+      </c>
+    </row>
+    <row r="10" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
         <v>0</v>
       </c>
@@ -779,7 +975,7 @@
         <v>8.9999999999999993E-3</v>
       </c>
       <c r="D10" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>85395.110202557713</v>
       </c>
       <c r="E10" s="4">
@@ -798,8 +994,34 @@
         <f t="shared" si="2"/>
         <v>10.216453251729327</v>
       </c>
-    </row>
-    <row r="11" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="K10" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="L10" s="1">
+        <v>8.9999999999999993E-3</v>
+      </c>
+      <c r="M10" s="4">
+        <f t="shared" si="5"/>
+        <v>85395.110202557713</v>
+      </c>
+      <c r="N10" s="4">
+        <f t="shared" si="6"/>
+        <v>768.55599182301933</v>
+      </c>
+      <c r="O10">
+        <f t="shared" si="3"/>
+        <v>85010.832206646213</v>
+      </c>
+      <c r="P10">
+        <f t="shared" si="7"/>
+        <v>872435.15131070488</v>
+      </c>
+      <c r="Q10">
+        <f t="shared" si="4"/>
+        <v>10.216453251729327</v>
+      </c>
+    </row>
+    <row r="11" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B11" s="3" t="s">
         <v>1</v>
       </c>
@@ -807,7 +1029,7 @@
         <v>0.01</v>
       </c>
       <c r="D11" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>84626.554210734699</v>
       </c>
       <c r="E11" s="4">
@@ -826,8 +1048,34 @@
         <f t="shared" si="2"/>
         <v>9.3046955113313068</v>
       </c>
-    </row>
-    <row r="12" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="K11" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="L11" s="1">
+        <v>0.01</v>
+      </c>
+      <c r="M11" s="4">
+        <f t="shared" si="5"/>
+        <v>84626.554210734699</v>
+      </c>
+      <c r="N11" s="4">
+        <f t="shared" si="6"/>
+        <v>846.26554210734696</v>
+      </c>
+      <c r="O11">
+        <f t="shared" si="3"/>
+        <v>84203.421439681028</v>
+      </c>
+      <c r="P11">
+        <f t="shared" si="7"/>
+        <v>787424.31910405867</v>
+      </c>
+      <c r="Q11">
+        <f t="shared" si="4"/>
+        <v>9.3046955113313068</v>
+      </c>
+    </row>
+    <row r="12" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B12" s="3" t="s">
         <v>2</v>
       </c>
@@ -835,7 +1083,7 @@
         <v>1.4E-2</v>
       </c>
       <c r="D12" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>83780.288668627356</v>
       </c>
       <c r="E12" s="4">
@@ -854,8 +1102,34 @@
         <f t="shared" si="2"/>
         <v>8.3936318296275836</v>
       </c>
-    </row>
-    <row r="13" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="K12" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="L12" s="1">
+        <v>1.4E-2</v>
+      </c>
+      <c r="M12" s="4">
+        <f t="shared" si="5"/>
+        <v>83780.288668627356</v>
+      </c>
+      <c r="N12" s="4">
+        <f t="shared" si="6"/>
+        <v>1172.9240413607829</v>
+      </c>
+      <c r="O12">
+        <f t="shared" si="3"/>
+        <v>83193.82664794696</v>
+      </c>
+      <c r="P12">
+        <f t="shared" si="7"/>
+        <v>703220.8976643777</v>
+      </c>
+      <c r="Q12">
+        <f t="shared" si="4"/>
+        <v>8.3936318296275836</v>
+      </c>
+    </row>
+    <row r="13" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
         <v>3</v>
       </c>
@@ -863,7 +1137,7 @@
         <v>1.0999999999999999E-2</v>
       </c>
       <c r="D13" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>82607.364627266579</v>
       </c>
       <c r="E13" s="4">
@@ -882,8 +1156,34 @@
         <f t="shared" si="2"/>
         <v>7.5057117947541423</v>
       </c>
-    </row>
-    <row r="14" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="K13" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="L13" s="1">
+        <v>1.0999999999999999E-2</v>
+      </c>
+      <c r="M13" s="4">
+        <f t="shared" si="5"/>
+        <v>82607.364627266579</v>
+      </c>
+      <c r="N13" s="4">
+        <f t="shared" si="6"/>
+        <v>908.68101089993229</v>
+      </c>
+      <c r="O13">
+        <f t="shared" si="3"/>
+        <v>82153.024121816619</v>
+      </c>
+      <c r="P13">
+        <f t="shared" si="7"/>
+        <v>620027.07101643085</v>
+      </c>
+      <c r="Q13">
+        <f t="shared" si="4"/>
+        <v>7.5057117947541423</v>
+      </c>
+    </row>
+    <row r="14" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B14" s="3" t="s">
         <v>4</v>
       </c>
@@ -891,7 +1191,7 @@
         <v>2.1000000000000001E-2</v>
       </c>
       <c r="D14" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>81698.683616366645</v>
       </c>
       <c r="E14" s="4">
@@ -910,8 +1210,34 @@
         <f t="shared" si="2"/>
         <v>6.5836317439374543</v>
       </c>
-    </row>
-    <row r="15" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="K14" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="L14" s="1">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="M14" s="4">
+        <f t="shared" si="5"/>
+        <v>81698.683616366645</v>
+      </c>
+      <c r="N14" s="4">
+        <f t="shared" si="6"/>
+        <v>1715.6723559436996</v>
+      </c>
+      <c r="O14">
+        <f t="shared" si="3"/>
+        <v>80840.847438394791</v>
+      </c>
+      <c r="P14">
+        <f t="shared" si="7"/>
+        <v>537874.04689461424</v>
+      </c>
+      <c r="Q14">
+        <f t="shared" si="4"/>
+        <v>6.5836317439374543</v>
+      </c>
+    </row>
+    <row r="15" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B15" s="3" t="s">
         <v>5</v>
       </c>
@@ -919,7 +1245,7 @@
         <v>3.1E-2</v>
       </c>
       <c r="D15" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>79983.011260422951</v>
       </c>
       <c r="E15" s="4">
@@ -938,8 +1264,34 @@
         <f t="shared" si="2"/>
         <v>5.7141284412027105</v>
       </c>
-    </row>
-    <row r="16" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="K15" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="L15" s="1">
+        <v>3.1E-2</v>
+      </c>
+      <c r="M15" s="4">
+        <f t="shared" si="5"/>
+        <v>79983.011260422951</v>
+      </c>
+      <c r="N15" s="4">
+        <f t="shared" si="6"/>
+        <v>2479.4733490731114</v>
+      </c>
+      <c r="O15">
+        <f t="shared" si="3"/>
+        <v>78743.274585886393</v>
+      </c>
+      <c r="P15">
+        <f t="shared" si="7"/>
+        <v>457033.19945621944</v>
+      </c>
+      <c r="Q15">
+        <f t="shared" si="4"/>
+        <v>5.7141284412027105</v>
+      </c>
+    </row>
+    <row r="16" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B16" s="3" t="s">
         <v>6</v>
       </c>
@@ -947,7 +1299,7 @@
         <v>5.0999999999999997E-2</v>
       </c>
       <c r="D16" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>77503.537911349835</v>
       </c>
       <c r="E16" s="4">
@@ -966,8 +1318,34 @@
         <f t="shared" si="2"/>
         <v>4.8809375038211682</v>
       </c>
-    </row>
-    <row r="17" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="K16" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="L16" s="1">
+        <v>5.0999999999999997E-2</v>
+      </c>
+      <c r="M16" s="4">
+        <f t="shared" si="5"/>
+        <v>77503.537911349835</v>
+      </c>
+      <c r="N16" s="4">
+        <f t="shared" si="6"/>
+        <v>3952.6804334788412</v>
+      </c>
+      <c r="O16">
+        <f t="shared" si="3"/>
+        <v>75527.197694610411</v>
+      </c>
+      <c r="P16">
+        <f t="shared" si="7"/>
+        <v>378289.92487033311</v>
+      </c>
+      <c r="Q16">
+        <f t="shared" si="4"/>
+        <v>4.8809375038211682</v>
+      </c>
+    </row>
+    <row r="17" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B17" s="3" t="s">
         <v>7</v>
       </c>
@@ -975,7 +1353,7 @@
         <v>5.8999999999999997E-2</v>
       </c>
       <c r="D17" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>73550.857477870988</v>
       </c>
       <c r="E17" s="4">
@@ -994,8 +1372,34 @@
         <f t="shared" si="2"/>
         <v>4.1163725013921679</v>
       </c>
-    </row>
-    <row r="18" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="K17" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="L17" s="1">
+        <v>5.8999999999999997E-2</v>
+      </c>
+      <c r="M17" s="4">
+        <f t="shared" si="5"/>
+        <v>73550.857477870988</v>
+      </c>
+      <c r="N17" s="4">
+        <f t="shared" si="6"/>
+        <v>4339.5005911943881</v>
+      </c>
+      <c r="O17">
+        <f t="shared" si="3"/>
+        <v>71381.107182273787</v>
+      </c>
+      <c r="P17">
+        <f t="shared" si="7"/>
+        <v>302762.72717572266</v>
+      </c>
+      <c r="Q17">
+        <f t="shared" si="4"/>
+        <v>4.1163725013921679</v>
+      </c>
+    </row>
+    <row r="18" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B18" s="3" t="s">
         <v>8</v>
       </c>
@@ -1003,7 +1407,7 @@
         <v>8.8999999999999996E-2</v>
       </c>
       <c r="D18" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>69211.3568866766</v>
       </c>
       <c r="E18" s="4">
@@ -1022,8 +1426,34 @@
         <f t="shared" si="2"/>
         <v>3.3431163670479997</v>
       </c>
-    </row>
-    <row r="19" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="K18" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="L18" s="1">
+        <v>8.8999999999999996E-2</v>
+      </c>
+      <c r="M18" s="4">
+        <f t="shared" si="5"/>
+        <v>69211.3568866766</v>
+      </c>
+      <c r="N18" s="4">
+        <f t="shared" si="6"/>
+        <v>6159.8107629142169</v>
+      </c>
+      <c r="O18">
+        <f t="shared" si="3"/>
+        <v>66131.451505219491</v>
+      </c>
+      <c r="P18">
+        <f t="shared" si="7"/>
+        <v>231381.6199934489</v>
+      </c>
+      <c r="Q18">
+        <f t="shared" si="4"/>
+        <v>3.3431163670480006</v>
+      </c>
+    </row>
+    <row r="19" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B19" s="3" t="s">
         <v>9</v>
       </c>
@@ -1031,7 +1461,7 @@
         <v>0.11700000000000001</v>
       </c>
       <c r="D19" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>63051.546123762382</v>
       </c>
       <c r="E19" s="4">
@@ -1050,8 +1480,34 @@
         <f t="shared" si="2"/>
         <v>2.6208741680000007</v>
       </c>
-    </row>
-    <row r="20" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="K19" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="L19" s="1">
+        <v>0.11700000000000001</v>
+      </c>
+      <c r="M19" s="4">
+        <f t="shared" si="5"/>
+        <v>63051.546123762382</v>
+      </c>
+      <c r="N19" s="4">
+        <f t="shared" si="6"/>
+        <v>7377.0308964801989</v>
+      </c>
+      <c r="O19">
+        <f t="shared" si="3"/>
+        <v>59363.030675522285</v>
+      </c>
+      <c r="P19">
+        <f t="shared" si="7"/>
+        <v>165250.16848822939</v>
+      </c>
+      <c r="Q19">
+        <f t="shared" si="4"/>
+        <v>2.6208741680000007</v>
+      </c>
+    </row>
+    <row r="20" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B20" s="3" t="s">
         <v>10</v>
       </c>
@@ -1059,7 +1515,7 @@
         <v>0.19800000000000001</v>
       </c>
       <c r="D20" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>55674.515227282187</v>
       </c>
       <c r="E20" s="4">
@@ -1078,8 +1534,34 @@
         <f t="shared" si="2"/>
         <v>1.901896</v>
       </c>
-    </row>
-    <row r="21" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="K20" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="L20" s="1">
+        <v>0.19800000000000001</v>
+      </c>
+      <c r="M20" s="4">
+        <f t="shared" si="5"/>
+        <v>55674.515227282187</v>
+      </c>
+      <c r="N20" s="4">
+        <f t="shared" si="6"/>
+        <v>11023.554015001873</v>
+      </c>
+      <c r="O20">
+        <f t="shared" si="3"/>
+        <v>50162.738219781255</v>
+      </c>
+      <c r="P20">
+        <f t="shared" si="7"/>
+        <v>105887.13781270708</v>
+      </c>
+      <c r="Q20">
+        <f t="shared" si="4"/>
+        <v>1.901896</v>
+      </c>
+    </row>
+    <row r="21" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B21" s="3" t="s">
         <v>11</v>
       </c>
@@ -1087,7 +1569,7 @@
         <v>0.252</v>
       </c>
       <c r="D21" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>44650.961212280316</v>
       </c>
       <c r="E21" s="4">
@@ -1106,8 +1588,34 @@
         <f t="shared" si="2"/>
         <v>1.248</v>
       </c>
-    </row>
-    <row r="22" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="K21" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="L21" s="1">
+        <v>0.252</v>
+      </c>
+      <c r="M21" s="4">
+        <f t="shared" si="5"/>
+        <v>44650.961212280316</v>
+      </c>
+      <c r="N21" s="4">
+        <f t="shared" si="6"/>
+        <v>11252.042225494639</v>
+      </c>
+      <c r="O21">
+        <f t="shared" si="3"/>
+        <v>39024.940099532992</v>
+      </c>
+      <c r="P21">
+        <f t="shared" si="7"/>
+        <v>55724.399592925831</v>
+      </c>
+      <c r="Q21">
+        <f t="shared" si="4"/>
+        <v>1.248</v>
+      </c>
+    </row>
+    <row r="22" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B22" s="3" t="s">
         <v>12</v>
       </c>
@@ -1115,7 +1623,7 @@
         <v>1</v>
       </c>
       <c r="D22" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="8"/>
         <v>33398.918986785677</v>
       </c>
       <c r="E22" s="4">
@@ -1123,7 +1631,7 @@
         <v>33398.918986785677</v>
       </c>
       <c r="F22">
-        <f t="shared" si="1"/>
+        <f>D22-(E22/2)</f>
         <v>16699.459493392838</v>
       </c>
       <c r="G22">
@@ -1131,7 +1639,33 @@
         <v>16699.459493392838</v>
       </c>
       <c r="H22">
-        <f t="shared" si="2"/>
+        <f>G22/D22</f>
+        <v>0.5</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="L22" s="1">
+        <v>1</v>
+      </c>
+      <c r="M22" s="4">
+        <f t="shared" si="5"/>
+        <v>33398.918986785677</v>
+      </c>
+      <c r="N22" s="4">
+        <f t="shared" si="6"/>
+        <v>33398.918986785677</v>
+      </c>
+      <c r="O22">
+        <f t="shared" si="3"/>
+        <v>16699.459493392838</v>
+      </c>
+      <c r="P22">
+        <f t="shared" si="7"/>
+        <v>16699.459493392838</v>
+      </c>
+      <c r="Q22">
+        <f t="shared" si="4"/>
         <v>0.5</v>
       </c>
     </row>
@@ -1141,19 +1675,19 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1B8DF6A-CEF7-436F-B4BF-B3CEA03AA66E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="13.54296875" customWidth="1"/>
-    <col min="4" max="4" width="10.90625" customWidth="1"/>
-    <col min="5" max="5" width="14.81640625" customWidth="1"/>
-    <col min="6" max="6" width="15.36328125" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" customWidth="1"/>
+    <col min="4" max="4" width="10.85546875" customWidth="1"/>
+    <col min="5" max="5" width="14.85546875" customWidth="1"/>
+    <col min="6" max="6" width="15.42578125" customWidth="1"/>
     <col min="7" max="7" width="15" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
     <col min="9" max="9" width="13" customWidth="1"/>
     <col min="10" max="10" width="12" customWidth="1"/>
-    <col min="11" max="11" width="10.81640625" customWidth="1"/>
+    <col min="11" max="11" width="10.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.35">

</xml_diff>